<commit_message>
fix(cost-plan): prioritize original order tag in root section sorting v3.7.28
</commit_message>
<xml_diff>
--- a/documents/2.Phụ lục 01 Bảng giá HĐ TSM_HGP - TBA 110kV Phước Lý.xlsx
+++ b/documents/2.Phụ lục 01 Bảng giá HĐ TSM_HGP - TBA 110kV Phước Lý.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BCCF732-BCD4-448B-B1EC-37742EA4BDE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9D7502E-A8D9-41C6-9384-9707BDB8BDE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Scada_TTLL" sheetId="1" r:id="rId1"/>
@@ -24,8 +24,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -474,9 +472,6 @@
     <t>Ống bảo vệ cáp quang HDPE F32, bao gồm trọn bộ phụ kiện lắp đặt hoàn chỉnh</t>
   </si>
   <si>
-    <t>PHẦN CÀI ĐẶT, CẤU HÌNH VÀ THÍ NGHIỆM HIỆU CHỈNH ĐỂ HOÀN CHỈNH KẾT NỐI HỆ THỐNG DỮ LIỆU SCADA CỦA RƠ LE F87L LẮP MỚI TẠI NGĂN LỘ 176 TẠI TBA 220kV CẦN ĐƯỚC VỀ CÁC TRUNG TÂM ĐIỀU ĐỘ SSO, EVNSPC VÀ ĐIỆN LỰC ĐỊA PHƯƠNG - DO NHÀ THẦU THỰC HIỆN (BAO GỒM CÔNG TÁC CÀI ĐẶT,CẤU HÌNH TẠI SSO, EVNSPC VÀ ĐIỆN LỰC ĐỊA PHƯƠNG)</t>
-  </si>
-  <si>
     <t>CẤU HÌNH VÀ CÀI ĐẶT DỮ LIỆU SCADA TRÊN HỆ THỐNG MÁY CHỦ SCADA/EMS TẠI TRUNG TÂM ĐIỀU ĐỘ HỆ THỐNG ĐIỆN MIỀN NAM (SSO) CHO TBA 110kV PHƯỚC LÝ - DO NHÀ THẦU THỰC HIỆN</t>
   </si>
   <si>
@@ -532,6 +527,9 @@
   </si>
   <si>
     <t>(Bằng chữ: Một tỷ, sáu trăm lẻ tám triệu, bốn trăm bảy mươi mốt nghìn đồng./.)</t>
+  </si>
+  <si>
+    <t>CẤU HÌNH VÀ THÍ NGHIỆM HIỆU CHỈNH ĐỂ HOÀN CHỈNH KẾT NỐI HỆ THỐNG DỮ LIỆU SCADA CỦA RƠ LE F87L LẮP MỚI TẠI NGĂN LỘ 176 TẠI TBA 220kV CẦN ĐƯỚC VỀ CÁC TRUNG TÂM ĐIỀU ĐỘ SSO, EVNSPC VÀ ĐIỆN LỰC ĐỊA PHƯƠNG - DO NHÀ THẦU THỰC HIỆN (BAO GỒM CÔNG TÁC CÀI ĐẶT,CẤU HÌNH TẠI SSO, EVNSPC VÀ ĐIỆN LỰC ĐỊA PHƯƠNG)</t>
   </si>
 </sst>
 </file>
@@ -539,10 +537,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
-    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="164" formatCode="_-* #,##0.00\ _₫_-;\-* #,##0.00\ _₫_-;_-* &quot;-&quot;??\ _₫_-;_-@_-"/>
-    <numFmt numFmtId="165" formatCode="_-* #,##0\ _₫_-;\-* #,##0\ _₫_-;_-* &quot;-&quot;??\ _₫_-;_-@_-"/>
-    <numFmt numFmtId="166" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="_-* #,##0.00\ _₫_-;\-* #,##0.00\ _₫_-;_-* &quot;-&quot;??\ _₫_-;_-@_-"/>
+    <numFmt numFmtId="166" formatCode="_-* #,##0\ _₫_-;\-* #,##0\ _₫_-;_-* &quot;-&quot;??\ _₫_-;_-@_-"/>
+    <numFmt numFmtId="167" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="21" x14ac:knownFonts="1">
     <font>
@@ -798,9 +796,9 @@
   </borders>
   <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="100">
@@ -814,25 +812,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="11" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="11" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="15" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -853,10 +851,10 @@
     <xf numFmtId="10" fontId="11" fillId="3" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="0" fillId="3" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -892,7 +890,7 @@
     <xf numFmtId="3" fontId="15" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -901,19 +899,19 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="43" fontId="2" fillId="4" borderId="3" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="4" borderId="3" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="4" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="10" fillId="4" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="4" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="10" fillId="4" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="4" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="10" fillId="4" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="4" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="10" fillId="4" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -925,7 +923,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="43" fontId="2" fillId="0" borderId="2" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -934,10 +932,10 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="4" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="10" fillId="4" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="4" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="10" fillId="4" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="10" fillId="4" borderId="2" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -952,7 +950,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="2" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="2" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -961,7 +959,7 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="4" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="6" fillId="4" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="6" fillId="4" borderId="2" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -973,10 +971,10 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="43" fontId="3" fillId="4" borderId="2" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="2" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="4" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="4" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -994,10 +992,10 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="43" fontId="2" fillId="4" borderId="2" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="4" borderId="2" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="6" fillId="4" borderId="2" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="2" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1012,16 +1010,16 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="4" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="4" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="4" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="6" fillId="4" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="4" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="6" fillId="4" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="6" fillId="4" borderId="4" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1042,16 +1040,16 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="43" fontId="3" fillId="4" borderId="5" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="5" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="4" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="4" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="4" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="6" fillId="4" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="4" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="6" fillId="4" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1063,24 +1061,36 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="43" fontId="2" fillId="4" borderId="5" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="4" borderId="5" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="4" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="10" fillId="4" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="4" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="10" fillId="4" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="4" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="10" fillId="4" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="4" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="10" fillId="4" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="4" fontId="10" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="16" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1088,18 +1098,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="10" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="16" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1482,68 +1480,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="93" t="s">
+      <c r="A1" s="97" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="93"/>
-      <c r="C1" s="93"/>
-      <c r="D1" s="93"/>
-      <c r="E1" s="93"/>
-      <c r="F1" s="93"/>
-      <c r="G1" s="93"/>
-      <c r="H1" s="93"/>
-      <c r="I1" s="93"/>
-      <c r="J1" s="93"/>
-      <c r="K1" s="93"/>
-      <c r="L1" s="93"/>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
+      <c r="K1" s="97"/>
+      <c r="L1" s="97"/>
     </row>
     <row r="2" spans="1:12" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="94" t="s">
+      <c r="A2" s="98" t="s">
         <v>24</v>
       </c>
-      <c r="B2" s="94"/>
-      <c r="C2" s="94"/>
-      <c r="D2" s="94"/>
-      <c r="E2" s="94"/>
-      <c r="F2" s="94"/>
-      <c r="G2" s="94"/>
-      <c r="H2" s="94"/>
-      <c r="I2" s="94"/>
-      <c r="J2" s="94"/>
-      <c r="K2" s="94"/>
-      <c r="L2" s="94"/>
+      <c r="B2" s="98"/>
+      <c r="C2" s="98"/>
+      <c r="D2" s="98"/>
+      <c r="E2" s="98"/>
+      <c r="F2" s="98"/>
+      <c r="G2" s="98"/>
+      <c r="H2" s="98"/>
+      <c r="I2" s="98"/>
+      <c r="J2" s="98"/>
+      <c r="K2" s="98"/>
+      <c r="L2" s="98"/>
     </row>
     <row r="3" spans="1:12" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="94" t="s">
+      <c r="A3" s="98" t="s">
         <v>25</v>
       </c>
-      <c r="B3" s="94"/>
-      <c r="C3" s="94"/>
-      <c r="D3" s="94"/>
-      <c r="E3" s="94"/>
-      <c r="F3" s="94"/>
-      <c r="G3" s="94"/>
-      <c r="H3" s="94"/>
-      <c r="I3" s="94"/>
-      <c r="J3" s="94"/>
-      <c r="K3" s="94"/>
-      <c r="L3" s="94"/>
+      <c r="B3" s="98"/>
+      <c r="C3" s="98"/>
+      <c r="D3" s="98"/>
+      <c r="E3" s="98"/>
+      <c r="F3" s="98"/>
+      <c r="G3" s="98"/>
+      <c r="H3" s="98"/>
+      <c r="I3" s="98"/>
+      <c r="J3" s="98"/>
+      <c r="K3" s="98"/>
+      <c r="L3" s="98"/>
     </row>
     <row r="4" spans="1:12" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="95" t="s">
+      <c r="A4" s="99" t="s">
         <v>26</v>
       </c>
-      <c r="B4" s="95"/>
-      <c r="C4" s="95"/>
-      <c r="D4" s="95"/>
-      <c r="E4" s="95"/>
-      <c r="F4" s="95"/>
-      <c r="G4" s="95"/>
-      <c r="H4" s="95"/>
-      <c r="I4" s="95"/>
-      <c r="J4" s="95"/>
-      <c r="K4" s="95"/>
-      <c r="L4" s="95"/>
+      <c r="B4" s="99"/>
+      <c r="C4" s="99"/>
+      <c r="D4" s="99"/>
+      <c r="E4" s="99"/>
+      <c r="F4" s="99"/>
+      <c r="G4" s="99"/>
+      <c r="H4" s="99"/>
+      <c r="I4" s="99"/>
+      <c r="J4" s="99"/>
+      <c r="K4" s="99"/>
+      <c r="L4" s="99"/>
     </row>
     <row r="5" spans="1:12" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A5" s="20"/>
@@ -1560,58 +1558,58 @@
       <c r="L5" s="22"/>
     </row>
     <row r="6" spans="1:12" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="96" t="s">
+      <c r="A6" s="95" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="96" t="s">
+      <c r="B6" s="95" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="96" t="s">
+      <c r="C6" s="95" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="96" t="s">
+      <c r="D6" s="95" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="96" t="s">
+      <c r="E6" s="95" t="s">
         <v>3</v>
       </c>
-      <c r="F6" s="96" t="s">
+      <c r="F6" s="95" t="s">
         <v>4</v>
       </c>
-      <c r="G6" s="96" t="s">
+      <c r="G6" s="95" t="s">
         <v>5</v>
       </c>
-      <c r="H6" s="96" t="s">
+      <c r="H6" s="95" t="s">
         <v>10</v>
       </c>
-      <c r="I6" s="96" t="s">
+      <c r="I6" s="95" t="s">
         <v>11</v>
       </c>
-      <c r="J6" s="96"/>
-      <c r="K6" s="96" t="s">
+      <c r="J6" s="95"/>
+      <c r="K6" s="95" t="s">
         <v>14</v>
       </c>
-      <c r="L6" s="99" t="s">
+      <c r="L6" s="96" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="96"/>
-      <c r="B7" s="96"/>
-      <c r="C7" s="96"/>
-      <c r="D7" s="96"/>
-      <c r="E7" s="96"/>
-      <c r="F7" s="96"/>
-      <c r="G7" s="96"/>
-      <c r="H7" s="96"/>
+      <c r="A7" s="95"/>
+      <c r="B7" s="95"/>
+      <c r="C7" s="95"/>
+      <c r="D7" s="95"/>
+      <c r="E7" s="95"/>
+      <c r="F7" s="95"/>
+      <c r="G7" s="95"/>
+      <c r="H7" s="95"/>
       <c r="I7" s="23" t="s">
         <v>12</v>
       </c>
       <c r="J7" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="K7" s="96"/>
-      <c r="L7" s="99"/>
+      <c r="K7" s="95"/>
+      <c r="L7" s="96"/>
     </row>
     <row r="8" spans="1:12" s="5" customFormat="1" ht="99" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="31">
@@ -1648,7 +1646,7 @@
         <v>1</v>
       </c>
       <c r="D9" s="78" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E9" s="81"/>
       <c r="F9" s="81"/>
@@ -1683,7 +1681,7 @@
         <v>1</v>
       </c>
       <c r="D10" s="78" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E10" s="81"/>
       <c r="F10" s="81"/>
@@ -1718,7 +1716,7 @@
         <v>1</v>
       </c>
       <c r="D11" s="78" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E11" s="81"/>
       <c r="F11" s="81"/>
@@ -1753,7 +1751,7 @@
         <v>1</v>
       </c>
       <c r="D12" s="78" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E12" s="81"/>
       <c r="F12" s="81"/>
@@ -1788,7 +1786,7 @@
         <v>2</v>
       </c>
       <c r="D13" s="78" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E13" s="81"/>
       <c r="F13" s="81"/>
@@ -1823,7 +1821,7 @@
         <v>1</v>
       </c>
       <c r="D14" s="78" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E14" s="81"/>
       <c r="F14" s="81"/>
@@ -1858,7 +1856,7 @@
         <v>1</v>
       </c>
       <c r="D15" s="78" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E15" s="81"/>
       <c r="F15" s="81"/>
@@ -1915,7 +1913,7 @@
         <v>1</v>
       </c>
       <c r="D17" s="78" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E17" s="81"/>
       <c r="F17" s="81"/>
@@ -1950,7 +1948,7 @@
         <v>5</v>
       </c>
       <c r="D18" s="78" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E18" s="81"/>
       <c r="F18" s="81"/>
@@ -1985,7 +1983,7 @@
         <v>1</v>
       </c>
       <c r="D19" s="78" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E19" s="81"/>
       <c r="F19" s="81"/>
@@ -2020,7 +2018,7 @@
         <v>1</v>
       </c>
       <c r="D20" s="78" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E20" s="81"/>
       <c r="F20" s="81"/>
@@ -2055,7 +2053,7 @@
         <v>1</v>
       </c>
       <c r="D21" s="78" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E21" s="81"/>
       <c r="F21" s="81"/>
@@ -2090,7 +2088,7 @@
         <v>1</v>
       </c>
       <c r="D22" s="78" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E22" s="81"/>
       <c r="F22" s="81"/>
@@ -2125,7 +2123,7 @@
         <v>1</v>
       </c>
       <c r="D23" s="78" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E23" s="81"/>
       <c r="F23" s="81"/>
@@ -2185,10 +2183,10 @@
         <v>19</v>
       </c>
       <c r="E25" s="81" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F25" s="81" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="G25" s="82">
         <v>90776000</v>
@@ -2221,13 +2219,13 @@
         <v>1</v>
       </c>
       <c r="D26" s="78" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E26" s="81" t="s">
+        <v>162</v>
+      </c>
+      <c r="F26" s="81" t="s">
         <v>163</v>
-      </c>
-      <c r="F26" s="81" t="s">
-        <v>164</v>
       </c>
       <c r="G26" s="82">
         <v>123455000</v>
@@ -2260,13 +2258,13 @@
         <v>1</v>
       </c>
       <c r="D27" s="78" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E27" s="81" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F27" s="81" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G27" s="82">
         <v>302585000</v>
@@ -2303,7 +2301,7 @@
       </c>
       <c r="E28" s="81"/>
       <c r="F28" s="81" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G28" s="82">
         <v>12708500</v>
@@ -2340,7 +2338,7 @@
       </c>
       <c r="E29" s="81"/>
       <c r="F29" s="81" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G29" s="82">
         <v>12708667</v>
@@ -2377,7 +2375,7 @@
       </c>
       <c r="E30" s="81"/>
       <c r="F30" s="81" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G30" s="82">
         <v>8472333</v>
@@ -2410,13 +2408,13 @@
         <v>120</v>
       </c>
       <c r="D31" s="78" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E31" s="81" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F31" s="81" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="G31" s="82">
         <v>30258</v>
@@ -2449,7 +2447,7 @@
         <v>10</v>
       </c>
       <c r="D32" s="78" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E32" s="81" t="s">
         <v>21</v>
@@ -2488,7 +2486,7 @@
         <v>2</v>
       </c>
       <c r="D33" s="78" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E33" s="81" t="s">
         <v>21</v>
@@ -2527,7 +2525,7 @@
         <v>2</v>
       </c>
       <c r="D34" s="78" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E34" s="81" t="s">
         <v>21</v>
@@ -2566,11 +2564,11 @@
         <v>100</v>
       </c>
       <c r="D35" s="78" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E35" s="81"/>
       <c r="F35" s="81" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G35" s="82">
         <v>42360</v>
@@ -2603,11 +2601,11 @@
         <v>6</v>
       </c>
       <c r="D36" s="78" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E36" s="81"/>
       <c r="F36" s="81" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G36" s="82">
         <v>30333</v>
@@ -2640,7 +2638,7 @@
         <v>10</v>
       </c>
       <c r="D37" s="78" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E37" s="81"/>
       <c r="F37" s="30" t="s">
@@ -2677,11 +2675,11 @@
         <v>100</v>
       </c>
       <c r="D38" s="78" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E38" s="81"/>
       <c r="F38" s="81" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G38" s="82">
         <v>78670</v>
@@ -2714,11 +2712,11 @@
         <v>100</v>
       </c>
       <c r="D39" s="78" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E39" s="81"/>
       <c r="F39" s="81" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G39" s="82">
         <v>66570</v>
@@ -2751,11 +2749,11 @@
         <v>2</v>
       </c>
       <c r="D40" s="78" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E40" s="81"/>
       <c r="F40" s="81" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G40" s="82">
         <v>3026000</v>
@@ -2788,11 +2786,11 @@
         <v>5</v>
       </c>
       <c r="D41" s="78" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E41" s="81"/>
       <c r="F41" s="81" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G41" s="82">
         <v>96800</v>
@@ -2829,7 +2827,7 @@
       </c>
       <c r="E42" s="81"/>
       <c r="F42" s="81" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G42" s="82">
         <v>6052000</v>
@@ -2884,13 +2882,13 @@
         <v>2</v>
       </c>
       <c r="D44" s="78" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E44" s="81" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F44" s="81" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G44" s="82">
         <v>4236000</v>
@@ -2923,11 +2921,11 @@
         <v>80</v>
       </c>
       <c r="D45" s="78" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E45" s="81"/>
       <c r="F45" s="81" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G45" s="82">
         <v>78675</v>
@@ -2960,11 +2958,11 @@
         <v>150</v>
       </c>
       <c r="D46" s="78" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E46" s="81"/>
       <c r="F46" s="81" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G46" s="82">
         <v>66567</v>
@@ -2997,7 +2995,7 @@
         <v>10</v>
       </c>
       <c r="D47" s="78" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E47" s="81"/>
       <c r="F47" s="30" t="s">
@@ -3034,7 +3032,7 @@
         <v>80</v>
       </c>
       <c r="D48" s="78" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E48" s="81"/>
       <c r="F48" s="30" t="s">
@@ -3071,7 +3069,7 @@
         <v>15</v>
       </c>
       <c r="D49" s="78" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E49" s="81"/>
       <c r="F49" s="30" t="s">
@@ -3108,11 +3106,11 @@
         <v>1</v>
       </c>
       <c r="D50" s="78" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E50" s="81"/>
       <c r="F50" s="81" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G50" s="82">
         <v>12103000</v>
@@ -3145,11 +3143,11 @@
         <v>1</v>
       </c>
       <c r="D51" s="78" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E51" s="81"/>
       <c r="F51" s="81" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G51" s="82">
         <v>6052000</v>
@@ -3182,7 +3180,7 @@
         <v>1</v>
       </c>
       <c r="D52" s="78" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E52" s="81"/>
       <c r="F52" s="30" t="s">
@@ -3241,13 +3239,13 @@
         <v>1</v>
       </c>
       <c r="D54" s="51" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E54" s="81" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F54" s="81" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="G54" s="53">
         <v>90776000</v>
@@ -3284,7 +3282,7 @@
       </c>
       <c r="E55" s="81"/>
       <c r="F55" s="81" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G55" s="53">
         <v>12709000</v>
@@ -3321,7 +3319,7 @@
       </c>
       <c r="E56" s="81"/>
       <c r="F56" s="81" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G56" s="53">
         <v>8472000</v>
@@ -3354,7 +3352,7 @@
         <v>6</v>
       </c>
       <c r="D57" s="48" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E57" s="59"/>
       <c r="F57" s="30" t="s">
@@ -3391,7 +3389,7 @@
         <v>2</v>
       </c>
       <c r="D58" s="48" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E58" s="52"/>
       <c r="F58" s="30" t="s">
@@ -3428,11 +3426,11 @@
         <v>50</v>
       </c>
       <c r="D59" s="48" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E59" s="77"/>
       <c r="F59" s="81" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G59" s="53">
         <v>66560</v>
@@ -3465,11 +3463,11 @@
         <v>6</v>
       </c>
       <c r="D60" s="48" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E60" s="58"/>
       <c r="F60" s="81" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G60" s="53">
         <v>2178667</v>
@@ -3502,7 +3500,7 @@
         <v>1</v>
       </c>
       <c r="D61" s="48" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E61" s="52"/>
       <c r="F61" s="52"/>
@@ -3559,13 +3557,13 @@
         <v>1</v>
       </c>
       <c r="D63" s="48" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E63" s="81" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F63" s="81" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="G63" s="53">
         <v>90776000</v>
@@ -3602,7 +3600,7 @@
       </c>
       <c r="E64" s="48"/>
       <c r="F64" s="81" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G64" s="53">
         <v>12708500</v>
@@ -3639,7 +3637,7 @@
       </c>
       <c r="E65" s="58"/>
       <c r="F65" s="81" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G65" s="53">
         <v>8472000</v>
@@ -3676,7 +3674,7 @@
       </c>
       <c r="E66" s="58"/>
       <c r="F66" s="81" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G66" s="53">
         <v>1208969</v>
@@ -3709,7 +3707,7 @@
         <v>8</v>
       </c>
       <c r="D67" s="48" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E67" s="58"/>
       <c r="F67" s="30" t="s">
@@ -3746,7 +3744,7 @@
         <v>1</v>
       </c>
       <c r="D68" s="48" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E68" s="48"/>
       <c r="F68" s="30" t="s">
@@ -3783,11 +3781,11 @@
         <v>50</v>
       </c>
       <c r="D69" s="48" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E69" s="48"/>
       <c r="F69" s="81" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G69" s="53">
         <v>66560</v>
@@ -3820,11 +3818,11 @@
         <v>6</v>
       </c>
       <c r="D70" s="48" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E70" s="58"/>
       <c r="F70" s="81" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G70" s="53">
         <v>2178667</v>
@@ -3857,7 +3855,7 @@
         <v>1</v>
       </c>
       <c r="D71" s="48" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E71" s="58"/>
       <c r="F71" s="30"/>
@@ -3914,7 +3912,7 @@
         <v>1</v>
       </c>
       <c r="D73" s="60" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E73" s="58" t="s">
         <v>23</v>
@@ -3953,13 +3951,13 @@
         <v>200</v>
       </c>
       <c r="D74" s="48" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E74" s="81" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F74" s="81" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="G74" s="53">
         <v>30260</v>
@@ -3992,7 +3990,7 @@
         <v>6</v>
       </c>
       <c r="D75" s="48" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E75" s="58"/>
       <c r="F75" s="30" t="s">
@@ -4029,7 +4027,7 @@
         <v>165</v>
       </c>
       <c r="D76" s="48" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E76" s="58"/>
       <c r="F76" s="30"/>
@@ -4064,7 +4062,7 @@
         <v>2</v>
       </c>
       <c r="D77" s="48" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E77" s="48"/>
       <c r="F77" s="30" t="s">
@@ -4101,11 +4099,11 @@
         <v>145</v>
       </c>
       <c r="D78" s="48" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E78" s="58"/>
       <c r="F78" s="81" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G78" s="53">
         <v>36310</v>
@@ -4132,7 +4130,7 @@
         <v>114</v>
       </c>
       <c r="B79" s="61" t="s">
-        <v>146</v>
+        <v>165</v>
       </c>
       <c r="C79" s="57">
         <v>1</v>
@@ -4169,13 +4167,13 @@
         <v>115</v>
       </c>
       <c r="B80" s="61" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C80" s="57">
         <v>1</v>
       </c>
       <c r="D80" s="48" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E80" s="58"/>
       <c r="F80" s="30" t="s">
@@ -4216,15 +4214,15 @@
       <c r="L81" s="75"/>
     </row>
     <row r="82" spans="1:12" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="97" t="s">
+      <c r="A82" s="93" t="s">
         <v>16</v>
       </c>
-      <c r="B82" s="97"/>
-      <c r="C82" s="97"/>
-      <c r="D82" s="97"/>
-      <c r="E82" s="97"/>
-      <c r="F82" s="97"/>
-      <c r="G82" s="97"/>
+      <c r="B82" s="93"/>
+      <c r="C82" s="93"/>
+      <c r="D82" s="93"/>
+      <c r="E82" s="93"/>
+      <c r="F82" s="93"/>
+      <c r="G82" s="93"/>
       <c r="H82" s="24"/>
       <c r="I82" s="25"/>
       <c r="J82" s="26"/>
@@ -4235,15 +4233,15 @@
       <c r="L82" s="27"/>
     </row>
     <row r="83" spans="1:12" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="97" t="s">
+      <c r="A83" s="93" t="s">
         <v>11</v>
       </c>
-      <c r="B83" s="97"/>
-      <c r="C83" s="97"/>
-      <c r="D83" s="97"/>
-      <c r="E83" s="97"/>
-      <c r="F83" s="97"/>
-      <c r="G83" s="97"/>
+      <c r="B83" s="93"/>
+      <c r="C83" s="93"/>
+      <c r="D83" s="93"/>
+      <c r="E83" s="93"/>
+      <c r="F83" s="93"/>
+      <c r="G83" s="93"/>
       <c r="H83" s="24"/>
       <c r="I83" s="25"/>
       <c r="J83" s="26"/>
@@ -4254,15 +4252,15 @@
       <c r="L83" s="27"/>
     </row>
     <row r="84" spans="1:12" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="97" t="s">
+      <c r="A84" s="93" t="s">
         <v>17</v>
       </c>
-      <c r="B84" s="97"/>
-      <c r="C84" s="97"/>
-      <c r="D84" s="97"/>
-      <c r="E84" s="97"/>
-      <c r="F84" s="97"/>
-      <c r="G84" s="97"/>
+      <c r="B84" s="93"/>
+      <c r="C84" s="93"/>
+      <c r="D84" s="93"/>
+      <c r="E84" s="93"/>
+      <c r="F84" s="93"/>
+      <c r="G84" s="93"/>
       <c r="H84" s="28"/>
       <c r="I84" s="28"/>
       <c r="J84" s="29"/>
@@ -4273,20 +4271,20 @@
       <c r="L84" s="27"/>
     </row>
     <row r="85" spans="1:12" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="98" t="s">
-        <v>165</v>
-      </c>
-      <c r="B85" s="98"/>
-      <c r="C85" s="98"/>
-      <c r="D85" s="98"/>
-      <c r="E85" s="98"/>
-      <c r="F85" s="98"/>
-      <c r="G85" s="98"/>
-      <c r="H85" s="98"/>
-      <c r="I85" s="98"/>
-      <c r="J85" s="98"/>
-      <c r="K85" s="98"/>
-      <c r="L85" s="98"/>
+      <c r="A85" s="94" t="s">
+        <v>164</v>
+      </c>
+      <c r="B85" s="94"/>
+      <c r="C85" s="94"/>
+      <c r="D85" s="94"/>
+      <c r="E85" s="94"/>
+      <c r="F85" s="94"/>
+      <c r="G85" s="94"/>
+      <c r="H85" s="94"/>
+      <c r="I85" s="94"/>
+      <c r="J85" s="94"/>
+      <c r="K85" s="94"/>
+      <c r="L85" s="94"/>
     </row>
     <row r="86" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E86" s="8"/>
@@ -4343,12 +4341,6 @@
   </sheetData>
   <autoFilter ref="A7:L80" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <mergeCells count="19">
-    <mergeCell ref="A82:G82"/>
-    <mergeCell ref="A84:G84"/>
-    <mergeCell ref="A83:G83"/>
-    <mergeCell ref="A85:L85"/>
-    <mergeCell ref="K6:K7"/>
-    <mergeCell ref="L6:L7"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="A3:L3"/>
@@ -4362,6 +4354,12 @@
     <mergeCell ref="G6:G7"/>
     <mergeCell ref="H6:H7"/>
     <mergeCell ref="I6:J6"/>
+    <mergeCell ref="A82:G82"/>
+    <mergeCell ref="A84:G84"/>
+    <mergeCell ref="A83:G83"/>
+    <mergeCell ref="A85:L85"/>
+    <mergeCell ref="K6:K7"/>
+    <mergeCell ref="L6:L7"/>
   </mergeCells>
   <phoneticPr fontId="18" type="noConversion"/>
   <conditionalFormatting sqref="H82:H83">

</xml_diff>